<commit_message>
Minor aesthetic tweak to remove visible righthand boarder from icon column.
</commit_message>
<xml_diff>
--- a/maturity matrix/maturity_matrix.xlsx
+++ b/maturity matrix/maturity_matrix.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charleshumble/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charleshumble/WebstormProjects/green-software-maturity-matrix/maturity matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{857A477A-394A-E64B-9196-35D63758262D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30DDABF9-94E5-FC4C-A247-0C5D331BCE3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -239,7 +239,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -275,11 +275,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFAAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFAAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFAAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -288,18 +301,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -945,27 +961,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="7"/>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8" t="s">
+      <c r="A1" s="5"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="6" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3"/>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="8" t="s">
         <v>5</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -985,8 +1001,8 @@
       </c>
     </row>
     <row r="3" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="5"/>
-      <c r="B3" s="6" t="s">
+      <c r="A3" s="4"/>
+      <c r="B3" s="9" t="s">
         <v>11</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -1007,7 +1023,7 @@
     </row>
     <row r="4" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3"/>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="8" t="s">
         <v>17</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -1027,8 +1043,8 @@
       </c>
     </row>
     <row r="5" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="5"/>
-      <c r="B5" s="6" t="s">
+      <c r="A5" s="4"/>
+      <c r="B5" s="9" t="s">
         <v>22</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -1049,7 +1065,7 @@
     </row>
     <row r="6" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3"/>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="8" t="s">
         <v>27</v>
       </c>
       <c r="C6" s="1" t="s">
@@ -1069,8 +1085,8 @@
       </c>
     </row>
     <row r="7" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="5"/>
-      <c r="B7" s="6" t="s">
+      <c r="A7" s="4"/>
+      <c r="B7" s="9" t="s">
         <v>31</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -1091,7 +1107,7 @@
     </row>
     <row r="8" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3"/>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="8" t="s">
         <v>36</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -1111,8 +1127,8 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="5"/>
-      <c r="B9" s="6" t="s">
+      <c r="A9" s="4"/>
+      <c r="B9" s="9" t="s">
         <v>41</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -1133,7 +1149,7 @@
     </row>
     <row r="10" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3"/>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="8" t="s">
         <v>45</v>
       </c>
       <c r="C10" s="1" t="s">

</xml_diff>

<commit_message>
Added first attempt at AI rows for discussion.
</commit_message>
<xml_diff>
--- a/maturity matrix/maturity_matrix.xlsx
+++ b/maturity matrix/maturity_matrix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charleshumble/WebstormProjects/green-software-maturity-matrix/maturity matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30DDABF9-94E5-FC4C-A247-0C5D331BCE3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F86A93E-7B6A-CA41-8D80-4F4FD27C8CC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Carbon Maturity Matrix" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="64">
   <si>
     <t>ASPIRING</t>
   </si>
@@ -176,6 +176,42 @@
   </si>
   <si>
     <t>demand shifting/shaping</t>
+  </si>
+  <si>
+    <t>Introduce "AI-Justification Gate"</t>
+  </si>
+  <si>
+    <t>Carbon-Intermittent Scheduling</t>
+  </si>
+  <si>
+    <t>Thermal Federated Learning</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Basic "Zombie" compute prevention via notebook auto-shutdowns.</t>
+  </si>
+  <si>
+    <t>AI training</t>
+  </si>
+  <si>
+    <t>AI Inferancing</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Strictly mandate all large-scale training jobs run only in regions with high Carbon-Free Energy.</t>
+  </si>
+  <si>
+    <t>Measure token use, know carbon cost/token.  Run workloads in multi-tenant hyperscale facilities with known, documented PUE and WUE metrics. If latency/data sovereignty rules allow run in locations with abundant green energy</t>
+  </si>
+  <si>
+    <t>Use sparse open weight models where possible/mixture of experts/Semantic casching. Actively wrk to minimise token use.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Model compression via Post-Training Distillation/Quantization/pruning. Apply demand shifting/shaping where latency allows</t>
+  </si>
+  <si>
+    <t>Fleetwide Cooptimization</t>
+  </si>
+  <si>
+    <t>Migrate baseline training to multi-tenant hyperscale facilities with known,  documented PUE and WUE metrics, in locations with abundant renewable energy.</t>
   </si>
 </sst>
 </file>
@@ -239,7 +275,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -288,11 +324,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFAAAAAA"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFAAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFAAAAAA"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -316,6 +372,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -948,14 +1013,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="65" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="38.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="22" customWidth="1"/>
   </cols>
@@ -1168,8 +1233,51 @@
         <v>50</v>
       </c>
     </row>
+    <row r="11" spans="1:7" ht="42" x14ac:dyDescent="0.2">
+      <c r="A11" s="4"/>
+      <c r="B11" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="84" x14ac:dyDescent="0.2">
+      <c r="A12" s="3"/>
+      <c r="B12" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adding DSAs.  Getting ready to invite comments.
</commit_message>
<xml_diff>
--- a/maturity matrix/maturity_matrix.xlsx
+++ b/maturity matrix/maturity_matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charleshumble/WebstormProjects/green-software-maturity-matrix/maturity matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F86A93E-7B6A-CA41-8D80-4F4FD27C8CC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80C0B189-53EE-BE42-997B-EF3BBD6EF5B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="40960" windowHeight="23040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Carbon Maturity Matrix" sheetId="1" r:id="rId1"/>
@@ -199,19 +199,19 @@
     <t xml:space="preserve"> Strictly mandate all large-scale training jobs run only in regions with high Carbon-Free Energy.</t>
   </si>
   <si>
-    <t>Measure token use, know carbon cost/token.  Run workloads in multi-tenant hyperscale facilities with known, documented PUE and WUE metrics. If latency/data sovereignty rules allow run in locations with abundant green energy</t>
-  </si>
-  <si>
-    <t>Use sparse open weight models where possible/mixture of experts/Semantic casching. Actively wrk to minimise token use.</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Model compression via Post-Training Distillation/Quantization/pruning. Apply demand shifting/shaping where latency allows</t>
   </si>
   <si>
     <t>Fleetwide Cooptimization</t>
   </si>
   <si>
-    <t>Migrate baseline training to multi-tenant hyperscale facilities with known,  documented PUE and WUE metrics, in locations with abundant renewable energy.</t>
+    <t>Use sparse open weight models where possible/mixture of experts/Semantic casching. Actively work to minimise token use.</t>
+  </si>
+  <si>
+    <t>Measure token use, know carbon cost/token.  Run workloads in multi-tenant hyperscale facilities with known, documented PUE and WUE metrics. If latency/data sovereignty rules allow run in locations with abundant green energy. Favour DSAs over CPUs</t>
+  </si>
+  <si>
+    <t>Migrate baseline training to multi-tenant hyperscale facilities with known,  documented PUE and WUE metrics, in locations with abundant renewable energy. Favour DSAs over CPUs</t>
   </si>
 </sst>
 </file>
@@ -1263,16 +1263,16 @@
         <v>52</v>
       </c>
       <c r="D12" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- Move matrix table from Excel to Word - Add new icons for each axis - Add Figma icon source file - Add PDF & PNG files
</commit_message>
<xml_diff>
--- a/maturity matrix/maturity_matrix.xlsx
+++ b/maturity matrix/maturity_matrix.xlsx
@@ -1,26 +1,142 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charleshumble/WebstormProjects/green-software-maturity-matrix/maturity matrix/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mark/Library/CloudStorage/Dropbox/Work/Projects/Conissaunce/green-software-maturity-matrix/maturity matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80C0B189-53EE-BE42-997B-EF3BBD6EF5B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9E51582-8CC8-854C-9E6B-6F13E9898CBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="40960" windowHeight="23040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="24300" windowHeight="24080" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Carbon Maturity Matrix" sheetId="1" r:id="rId1"/>
+    <sheet name="Carbon Maturity Matrix v2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="9">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="3"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="4"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="5"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="6"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="7"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="8"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="9">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+    <bk>
+      <rc t="1" v="1"/>
+    </bk>
+    <bk>
+      <rc t="1" v="2"/>
+    </bk>
+    <bk>
+      <rc t="1" v="3"/>
+    </bk>
+    <bk>
+      <rc t="1" v="4"/>
+    </bk>
+    <bk>
+      <rc t="1" v="5"/>
+    </bk>
+    <bk>
+      <rc t="1" v="6"/>
+    </bk>
+    <bk>
+      <rc t="1" v="7"/>
+    </bk>
+    <bk>
+      <rc t="1" v="8"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="118">
   <si>
     <t>ASPIRING</t>
   </si>
@@ -212,13 +328,178 @@
   </si>
   <si>
     <t>Migrate baseline training to multi-tenant hyperscale facilities with known,  documented PUE and WUE metrics, in locations with abundant renewable energy. Favour DSAs over CPUs</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Carbon neutral</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>Reducing per unit</t>
+  </si>
+  <si>
+    <t>Reducing absolutely</t>
+  </si>
+  <si>
+    <t>~ Zero</t>
+  </si>
+  <si>
+    <t>Predicted</t>
+  </si>
+  <si>
+    <t>Manual</t>
+  </si>
+  <si>
+    <t>Auto-rightsizing</t>
+  </si>
+  <si>
+    <t>Carbon SRE</t>
+  </si>
+  <si>
+    <t>Green hosting</t>
+  </si>
+  <si>
+    <t>Some targets</t>
+  </si>
+  <si>
+    <t>Rolling repair</t>
+  </si>
+  <si>
+    <t>Max orchestration</t>
+  </si>
+  <si>
+    <t>Edge integration</t>
+  </si>
+  <si>
+    <t>Carbon awareness</t>
+  </si>
+  <si>
+    <t>Feature tracking</t>
+  </si>
+  <si>
+    <t>Ad hoc</t>
+  </si>
+  <si>
+    <t>Basic / champions</t>
+  </si>
+  <si>
+    <t>Advanced</t>
+  </si>
+  <si>
+    <t>You're the leader</t>
+  </si>
+  <si>
+    <t>You're the trainer</t>
+  </si>
+  <si>
+    <t>All multi-tenant</t>
+  </si>
+  <si>
+    <t>AXIS</t>
+  </si>
+  <si>
+    <t>Commitments</t>
+  </si>
+  <si>
+    <t>Footprint</t>
+  </si>
+  <si>
+    <t>Metrics</t>
+  </si>
+  <si>
+    <t>Carbon ops</t>
+  </si>
+  <si>
+    <t>Energy</t>
+  </si>
+  <si>
+    <t>Devices</t>
+  </si>
+  <si>
+    <t>Utilization</t>
+  </si>
+  <si>
+    <t>Products</t>
+  </si>
+  <si>
+    <t>Training</t>
+  </si>
+  <si>
+    <t>Demand shifting / shaping</t>
+  </si>
+  <si>
+    <t>Feature carbon
+error budgets</t>
+  </si>
+  <si>
+    <t>Report scope 1 &amp; 2</t>
+  </si>
+  <si>
+    <t>Know scope 1 &amp; 2</t>
+  </si>
+  <si>
+    <t>Dynamic
+management</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>icon</t>
+  </si>
+  <si>
+    <t>10% offsets</t>
+  </si>
+  <si>
+    <t>1% offsets</t>
+  </si>
+  <si>
+    <t>Light-switch ops</t>
+  </si>
+  <si>
+    <t>10y - 90%</t>
+  </si>
+  <si>
+    <t>10y - 100%</t>
+  </si>
+  <si>
+    <t>Carbon zero
+with offsets</t>
+  </si>
+  <si>
+    <t>Layout notes</t>
+  </si>
+  <si>
+    <t>•</t>
+  </si>
+  <si>
+    <t>Icon images are placed in cells (Col B) so their size is controlled by Col B width</t>
+  </si>
+  <si>
+    <t>All cells (apart from icons) have left indent set</t>
+  </si>
+  <si>
+    <t>Font is Nunito to match GSF website and Maturity Matrix online docs</t>
+  </si>
+  <si>
+    <t>Table uses a Custom Table Style to control borders &amp; background colours (select cell, go to Table menu…)</t>
+  </si>
+  <si>
+    <t>Keep row heights consistent by adjusting all row heights simultaneously</t>
+  </si>
+  <si>
+    <t>Color reference from GSF website: Dark green = #006D69; Light green = #AECC53</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -246,8 +527,47 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Nunito Sans Normal"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Nunito Sans Normal"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Nunito Sans Normal"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Nunito Sans Normal SemiBold"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF006D69"/>
+      <name val="Nunito Sans Normal"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Nunito Sans Normal"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Nunito Sans Normal SemiBold"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -272,6 +592,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF009E9F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFAFDF3"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -348,7 +674,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -382,12 +708,450 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <dxfs count="24">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF2D2D2D"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Nunito Sans Normal"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" relativeIndent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF2D2D2D"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Nunito Sans Normal"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" relativeIndent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF2D2D2D"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Nunito Sans Normal"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" relativeIndent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF2D2D2D"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Nunito Sans Normal"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" relativeIndent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF2D2D2D"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Nunito Sans Normal"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" relativeIndent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Nunito Sans Normal SemiBold"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFAFDF3"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" relativeIndent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Nunito Sans Normal"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFAFDF3"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Nunito Sans Normal"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFAFDF3"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Nunito Sans Normal"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Nunito Sans Normal"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Nunito Sans Normal"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8F8F8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFA7C554"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="double">
+          <color theme="6"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FF006D69"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top/>
+        <bottom style="thick">
+          <color rgb="FFAECC53"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <color theme="1" tint="0.14996795556505021"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thick">
+          <color rgb="FF006D69"/>
+        </top>
+        <bottom style="thick">
+          <color rgb="FF006D69"/>
+        </bottom>
+        <vertical/>
+        <horizontal style="hair">
+          <color theme="0" tint="-0.14996795556505021"/>
+        </horizontal>
+      </border>
+    </dxf>
+  </dxfs>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Green Software Foundation" pivot="0" count="5" xr9:uid="{271AE576-60EB-0748-8E80-F19BB3F67D2B}">
+      <tableStyleElement type="wholeTable" dxfId="23"/>
+      <tableStyleElement type="headerRow" dxfId="22"/>
+      <tableStyleElement type="totalRow" dxfId="21"/>
+      <tableStyleElement type="firstColumn" dxfId="20"/>
+      <tableStyleElement type="firstRowStripe" dxfId="19"/>
+    </tableStyle>
+  </tableStyles>
+  <colors>
+    <mruColors>
+      <color rgb="FF006D69"/>
+      <color rgb="FFAECC53"/>
+      <color rgb="FFFAFDF3"/>
+      <color rgb="FFA7C554"/>
+      <color rgb="FFF8F8F8"/>
+      <color rgb="FF2E6C68"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -728,6 +1492,136 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="9">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>1</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>2</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>3</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>4</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>5</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>6</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>7</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>8</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+  <rel r:id="rId2"/>
+  <rel r:id="rId3"/>
+  <rel r:id="rId4"/>
+  <rel r:id="rId5"/>
+  <rel r:id="rId6"/>
+  <rel r:id="rId7"/>
+  <rel r:id="rId8"/>
+  <rel r:id="rId9"/>
+</richValueRels>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A64C7D79-7294-8145-964C-6A641ECE1365}" name="Table1" displayName="Table1" ref="B2:I11" headerRowDxfId="18" dataDxfId="17" totalsRowDxfId="16">
+  <autoFilter ref="B2:I11" xr:uid="{A64C7D79-7294-8145-964C-6A641ECE1365}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
+    <filterColumn colId="7" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="8">
+    <tableColumn id="8" xr3:uid="{C88E5E73-1337-274D-98FA-639F3884591F}" name="a" dataDxfId="15" totalsRowDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{538CFCEF-490C-2E44-9E80-C3C2F194BA4C}" name="icon" totalsRowLabel="Total" dataDxfId="13" totalsRowDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{C5505F4D-B7D3-1343-B3F1-AE209759E5A1}" name="AXIS" dataDxfId="11" totalsRowDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{BAB853F0-0E03-A144-A489-530BE7D9BD2B}" name="ASPIRING" dataDxfId="9" totalsRowDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{F20F6D69-B379-8547-896C-DA4AB63AB0B3}" name="AWARE" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{CD759EDE-074C-D342-83E9-57D1473117F6}" name="ACTING" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{F14F5DBD-40F0-084B-81B5-89427F234CB4}" name="AWESOME" dataDxfId="3" totalsRowDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{A6BF90E7-8AA9-D549-B4A1-413099998C11}" name="INSPIRING" totalsRowFunction="count" dataDxfId="1" totalsRowDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="Green Software Foundation" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1014,7 +1908,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
@@ -1025,7 +1919,7 @@
     <col min="7" max="7" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="36" customHeight="1">
       <c r="A1" s="5"/>
       <c r="B1" s="7"/>
       <c r="C1" s="6" t="s">
@@ -1044,7 +1938,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" ht="46" customHeight="1">
       <c r="A2" s="3"/>
       <c r="B2" s="8" t="s">
         <v>5</v>
@@ -1065,7 +1959,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" ht="46" customHeight="1">
       <c r="A3" s="4"/>
       <c r="B3" s="9" t="s">
         <v>11</v>
@@ -1086,7 +1980,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" ht="46" customHeight="1">
       <c r="A4" s="3"/>
       <c r="B4" s="8" t="s">
         <v>17</v>
@@ -1107,7 +2001,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="46" customHeight="1">
       <c r="A5" s="4"/>
       <c r="B5" s="9" t="s">
         <v>22</v>
@@ -1128,7 +2022,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" ht="46" customHeight="1">
       <c r="A6" s="3"/>
       <c r="B6" s="8" t="s">
         <v>27</v>
@@ -1149,7 +2043,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" ht="46" customHeight="1">
       <c r="A7" s="4"/>
       <c r="B7" s="9" t="s">
         <v>31</v>
@@ -1170,7 +2064,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" ht="46" customHeight="1">
       <c r="A8" s="3"/>
       <c r="B8" s="8" t="s">
         <v>36</v>
@@ -1191,7 +2085,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" ht="46" customHeight="1">
       <c r="A9" s="4"/>
       <c r="B9" s="9" t="s">
         <v>41</v>
@@ -1212,7 +2106,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" ht="46" customHeight="1">
       <c r="A10" s="3"/>
       <c r="B10" s="8" t="s">
         <v>45</v>
@@ -1233,7 +2127,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="42" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" ht="42">
       <c r="A11" s="4"/>
       <c r="B11" s="10" t="s">
         <v>56</v>
@@ -1254,7 +2148,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="84" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" ht="84">
       <c r="A12" s="3"/>
       <c r="B12" s="11" t="s">
         <v>57</v>
@@ -1280,4 +2174,328 @@
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{125542DC-B2ED-E04F-931B-7D8144F00270}">
+  <dimension ref="B1:I20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="1" width="4.6640625" style="16" customWidth="1"/>
+    <col min="2" max="2" width="1.5" style="23" customWidth="1"/>
+    <col min="3" max="3" width="3.83203125" style="16" customWidth="1"/>
+    <col min="4" max="4" width="14.1640625" style="25" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" style="19" customWidth="1"/>
+    <col min="6" max="9" width="22" style="19" customWidth="1"/>
+    <col min="10" max="10" width="19.6640625" style="16" customWidth="1"/>
+    <col min="11" max="16384" width="8.83203125" style="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:9" ht="32" customHeight="1">
+      <c r="C1" s="24"/>
+      <c r="D1" s="19"/>
+    </row>
+    <row r="2" spans="2:9" s="13" customFormat="1" ht="30" customHeight="1">
+      <c r="B2" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>103</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="E2" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="H2" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="I2" s="17" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" s="15" customFormat="1" ht="48" customHeight="1">
+      <c r="B3" s="14"/>
+      <c r="C3" s="21" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="E3" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="H3" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="I3" s="18" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" s="15" customFormat="1" ht="48" customHeight="1">
+      <c r="B4" s="14"/>
+      <c r="C4" s="14" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="G4" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="H4" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="I4" s="18" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" s="15" customFormat="1" ht="48" customHeight="1">
+      <c r="B5" s="14"/>
+      <c r="C5" s="14" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="E5" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="G5" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="H5" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="18" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" s="15" customFormat="1" ht="48" customHeight="1">
+      <c r="B6" s="14"/>
+      <c r="C6" s="14" t="e" vm="4">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="E6" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="F6" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="G6" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="H6" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="I6" s="18" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" s="15" customFormat="1" ht="48" customHeight="1">
+      <c r="B7" s="14"/>
+      <c r="C7" s="14" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="E7" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="F7" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="G7" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="H7" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="I7" s="18" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" s="15" customFormat="1" ht="48" customHeight="1">
+      <c r="B8" s="14"/>
+      <c r="C8" s="14" t="e" vm="6">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="F8" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="G8" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="H8" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="I8" s="18" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" s="15" customFormat="1" ht="48" customHeight="1">
+      <c r="B9" s="14"/>
+      <c r="C9" s="14" t="e" vm="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="E9" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="G9" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="H9" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="I9" s="18" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" s="15" customFormat="1" ht="48" customHeight="1">
+      <c r="B10" s="14"/>
+      <c r="C10" s="14" t="e" vm="8">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="E10" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="G10" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="H10" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="I10" s="18" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" s="15" customFormat="1" ht="48" customHeight="1">
+      <c r="B11" s="14"/>
+      <c r="C11" s="14" t="e" vm="9">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="G11" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="H11" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="I11" s="18" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9">
+      <c r="B14" s="26" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9">
+      <c r="C15" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="D15" s="23" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9">
+      <c r="C16" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" spans="3:4">
+      <c r="C17" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="18" spans="3:4">
+      <c r="C18" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="19" spans="3:4">
+      <c r="C19" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="20" spans="3:4">
+      <c r="C20" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>117</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>